<commit_message>
Version Packages: prepare 0.4.2 strong-beta release
</commit_message>
<xml_diff>
--- a/samples/visualization/geotech-viz-showcase.xlsx
+++ b/samples/visualization/geotech-viz-showcase.xlsx
@@ -7,13 +7,16 @@
     <sheet sheetId="1" name="settlement_profile" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="liquefaction_depth" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="pile_capacity_profile" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="compaction_curve" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="gradation_curve" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="cpt_profile" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>distance_m</t>
   </si>
@@ -49,6 +52,27 @@
   </si>
   <si>
     <t>cumulative_shaft_kn</t>
+  </si>
+  <si>
+    <t>moisture_content</t>
+  </si>
+  <si>
+    <t>dry_density_kn_m3</t>
+  </si>
+  <si>
+    <t>particle_size_mm</t>
+  </si>
+  <si>
+    <t>percent_passing</t>
+  </si>
+  <si>
+    <t>qc_mpa</t>
+  </si>
+  <si>
+    <t>fs_kpa</t>
+  </si>
+  <si>
+    <t>friction_ratio</t>
   </si>
 </sst>
 </file>
@@ -873,4 +897,283 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>16.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>18.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>19.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>16</v>
+      </c>
+      <c r="B6">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>18</v>
+      </c>
+      <c r="B7">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>20</v>
+      </c>
+      <c r="B8">
+        <v>18.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0.075</v>
+      </c>
+      <c r="B2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0.15</v>
+      </c>
+      <c r="B3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>0.3</v>
+      </c>
+      <c r="B4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>0.6</v>
+      </c>
+      <c r="B5">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1.18</v>
+      </c>
+      <c r="B6">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>2.36</v>
+      </c>
+      <c r="B7">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>4.75</v>
+      </c>
+      <c r="B8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>9.5</v>
+      </c>
+      <c r="B9">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>2.8</v>
+      </c>
+      <c r="C2">
+        <v>52</v>
+      </c>
+      <c r="D2">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>4.3</v>
+      </c>
+      <c r="C3">
+        <v>58</v>
+      </c>
+      <c r="D3">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>6.8</v>
+      </c>
+      <c r="C4">
+        <v>64</v>
+      </c>
+      <c r="D4">
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>8.9</v>
+      </c>
+      <c r="C5">
+        <v>71</v>
+      </c>
+      <c r="D5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>10.7</v>
+      </c>
+      <c r="C6">
+        <v>79</v>
+      </c>
+      <c r="D6">
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>12.9</v>
+      </c>
+      <c r="C7">
+        <v>86</v>
+      </c>
+      <c r="D7">
+        <v>0.67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>